<commit_message>
Preparing for and analysing HFR TDI ultrasound data.
</commit_message>
<xml_diff>
--- a/data/raw/2026-09-13_hfr-tdi-calibration-cases_codebook.xlsx
+++ b/data/raw/2026-09-13_hfr-tdi-calibration-cases_codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studntnu-my.sharepoint.com/personal/kjellhoy_ntnu_no/Documents/Documents/PhD/05_Analyse-i-R/Sharing-of-data-in-PhD-project/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="158" documentId="11_AD4DB114E441178AC67DF4C8DE97C310693EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90731C94-ABE0-4210-B767-DBA2914A82FC}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="11_AD4DB114E441178AC67DF4C8DE97C310693EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{542B7085-F26E-46F3-B14D-E1515888E120}"/>
   <bookViews>
-    <workbookView xWindow="-51705" yWindow="-13230" windowWidth="28695" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25905" yWindow="-2790" windowWidth="26010" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calibration codebook" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="198">
   <si>
     <t>Variable name</t>
   </si>
@@ -1374,6 +1374,12 @@
   </si>
   <si>
     <t>To be included in plax vs atypical plax comparison study</t>
+  </si>
+  <si>
+    <t>Leabe as "NA" if not uploaded, usually because of poor quality</t>
+  </si>
+  <si>
+    <t>File uploaded to FTP server but not optimal SW quality</t>
   </si>
 </sst>
 </file>
@@ -1881,7 +1887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" style="14" customWidth="1"/>
@@ -2272,790 +2278,801 @@
         <v>6</v>
       </c>
       <c r="C58" s="8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B59" s="6">
+        <v>7</v>
+      </c>
+      <c r="C59" s="8" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="14" t="s">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="B60" s="6">
+      <c r="B61" s="6">
         <v>1</v>
       </c>
-      <c r="C60" s="7" t="s">
+      <c r="C61" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D61" t="s">
         <v>176</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B61" s="6">
-        <v>2</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="D61" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B62" s="6">
+        <v>2</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D62" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B63" s="6">
         <v>3</v>
       </c>
-      <c r="C62" s="7" t="s">
+      <c r="C63" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D63" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B63" s="6"/>
-      <c r="C63" s="7"/>
-    </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="14" t="s">
+      <c r="B64" s="6"/>
+      <c r="C64" s="7"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B64" s="6">
+      <c r="B65" s="6">
         <v>1</v>
       </c>
-      <c r="C64" s="7" t="s">
+      <c r="C65" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="D64" t="s">
+      <c r="D65" t="s">
         <v>180</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B65" s="6">
-        <v>2</v>
-      </c>
-      <c r="C65" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="D65" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B66" s="6">
+        <v>2</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D66" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B67" s="6">
         <v>3</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="C67" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D66" t="s">
+      <c r="D67" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B67" s="6"/>
-      <c r="C67" s="7"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="14" t="s">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B68" s="6"/>
+      <c r="C68" s="7"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B69" s="6">
+      <c r="B70" s="6">
         <v>1</v>
       </c>
-      <c r="C69" s="8" t="s">
+      <c r="C70" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D70" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B70" s="6">
-        <v>2</v>
-      </c>
-      <c r="C70" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D70" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B71" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D71" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B72" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D72" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B73" s="6">
-        <v>5</v>
-      </c>
-      <c r="C73" s="28" t="s">
-        <v>47</v>
+        <v>4</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>45</v>
       </c>
       <c r="D73" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B74" s="6">
+        <v>5</v>
+      </c>
+      <c r="C74" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="D74" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B75" s="6">
         <v>6</v>
       </c>
-      <c r="C74" s="28" t="s">
+      <c r="C75" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D75" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B75" s="29">
-        <v>7</v>
-      </c>
-      <c r="C75" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D75" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B76" s="29">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D76" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B77" s="29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D77" s="30" t="s">
-        <v>56</v>
+        <v>53</v>
+      </c>
+      <c r="D77" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B78" s="29">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D78" t="s">
-        <v>58</v>
+        <v>55</v>
+      </c>
+      <c r="D78" s="30" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B79" s="29">
-        <v>11</v>
-      </c>
-      <c r="C79" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="D79" s="30" t="s">
-        <v>60</v>
+        <v>10</v>
+      </c>
+      <c r="C79" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D79" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B80" s="29">
+        <v>11</v>
+      </c>
+      <c r="C80" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="D80" s="30" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="81" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B81" s="29">
         <v>12</v>
       </c>
-      <c r="C80" s="28" t="s">
+      <c r="C81" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="D80" t="s">
+      <c r="D81" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="81" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B81" s="31">
-        <v>13</v>
-      </c>
-      <c r="C81" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="D81" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B82" s="31">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D82" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B83" s="31">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D83" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B84" s="31">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D84" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B85" s="31">
-        <v>17</v>
-      </c>
-      <c r="C85" s="28" t="s">
-        <v>71</v>
+        <v>16</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>69</v>
       </c>
       <c r="D85" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="86" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B86" s="31">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C86" s="28" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D86" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="87" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B87" s="31">
-        <v>19</v>
-      </c>
-      <c r="C87" s="8" t="s">
-        <v>75</v>
+        <v>18</v>
+      </c>
+      <c r="C87" s="28" t="s">
+        <v>73</v>
       </c>
       <c r="D87" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="88" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B88" s="31">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D88" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="89" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B89" s="31">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D89" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B90" s="31">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D90" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B91" s="31">
-        <v>23</v>
-      </c>
-      <c r="C91" s="28" t="s">
-        <v>83</v>
+        <v>22</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>81</v>
       </c>
       <c r="D91" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="92" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B92" s="31">
+        <v>23</v>
+      </c>
+      <c r="C92" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D92" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="93" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B93" s="31">
         <v>24</v>
       </c>
-      <c r="C92" s="28" t="s">
+      <c r="C93" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="D92" t="s">
+      <c r="D93" t="s">
         <v>86</v>
-      </c>
-    </row>
-    <row r="93" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B93" s="32">
-        <v>25</v>
-      </c>
-      <c r="C93" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D93" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B94" s="32">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D94" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B95" s="32">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="D95" s="30" t="s">
-        <v>92</v>
+        <v>89</v>
+      </c>
+      <c r="D95" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="96" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B96" s="32">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="D96" t="s">
-        <v>94</v>
+        <v>91</v>
+      </c>
+      <c r="D96" s="30" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B97" s="32">
-        <v>29</v>
-      </c>
-      <c r="C97" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="D97" s="30" t="s">
-        <v>96</v>
+        <v>28</v>
+      </c>
+      <c r="C97" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D97" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B98" s="32">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C98" s="28" t="s">
-        <v>97</v>
-      </c>
-      <c r="D98" t="s">
-        <v>98</v>
+        <v>95</v>
+      </c>
+      <c r="D98" s="30" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B99" s="32">
-        <v>31</v>
-      </c>
-      <c r="C99" s="8" t="s">
-        <v>99</v>
+        <v>30</v>
+      </c>
+      <c r="C99" s="28" t="s">
+        <v>97</v>
       </c>
       <c r="D99" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="100" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B100" s="32">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D100" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="101" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B101" s="32">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D101" s="30" t="s">
-        <v>104</v>
+        <v>101</v>
+      </c>
+      <c r="D101" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="102" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B102" s="32">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="D102" t="s">
-        <v>106</v>
+        <v>103</v>
+      </c>
+      <c r="D102" s="30" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="103" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B103" s="32">
-        <v>35</v>
-      </c>
-      <c r="C103" s="28" t="s">
-        <v>107</v>
-      </c>
-      <c r="D103" s="30" t="s">
-        <v>108</v>
+        <v>34</v>
+      </c>
+      <c r="C103" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D103" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="104" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B104" s="32">
+        <v>35</v>
+      </c>
+      <c r="C104" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D104" s="30" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="105" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B105" s="32">
         <v>36</v>
       </c>
-      <c r="C104" s="28" t="s">
+      <c r="C105" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="D104" t="s">
+      <c r="D105" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="105" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B105" s="33">
-        <v>37</v>
-      </c>
-      <c r="C105" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="D105" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="106" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B106" s="33">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D106" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="107" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B107" s="33">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="D107" s="30" t="s">
-        <v>116</v>
+        <v>113</v>
+      </c>
+      <c r="D107" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="108" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B108" s="33">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D108" t="s">
-        <v>118</v>
+        <v>115</v>
+      </c>
+      <c r="D108" s="30" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="109" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B109" s="33">
-        <v>41</v>
-      </c>
-      <c r="C109" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="D109" s="30" t="s">
-        <v>120</v>
+        <v>40</v>
+      </c>
+      <c r="C109" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="D109" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="110" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B110" s="33">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C110" s="28" t="s">
-        <v>121</v>
-      </c>
-      <c r="D110" t="s">
-        <v>122</v>
+        <v>119</v>
+      </c>
+      <c r="D110" s="30" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="111" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B111" s="33">
-        <v>43</v>
-      </c>
-      <c r="C111" s="8" t="s">
-        <v>123</v>
+        <v>42</v>
+      </c>
+      <c r="C111" s="28" t="s">
+        <v>121</v>
       </c>
       <c r="D111" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="112" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B112" s="33">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C112" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D112" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="113" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B113" s="33">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="D113" s="30" t="s">
-        <v>128</v>
+        <v>125</v>
+      </c>
+      <c r="D113" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="114" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B114" s="33">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="D114" t="s">
-        <v>130</v>
+        <v>127</v>
+      </c>
+      <c r="D114" s="30" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="115" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B115" s="33">
-        <v>47</v>
-      </c>
-      <c r="C115" s="28" t="s">
-        <v>131</v>
-      </c>
-      <c r="D115" s="30" t="s">
-        <v>132</v>
+        <v>46</v>
+      </c>
+      <c r="C115" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="D115" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="116" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B116" s="33">
+        <v>47</v>
+      </c>
+      <c r="C116" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="D116" s="30" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="117" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B117" s="33">
         <v>48</v>
       </c>
-      <c r="C116" s="28" t="s">
+      <c r="C117" s="28" t="s">
         <v>133</v>
       </c>
-      <c r="D116" t="s">
+      <c r="D117" t="s">
         <v>134</v>
-      </c>
-    </row>
-    <row r="117" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B117" s="31">
-        <v>49</v>
-      </c>
-      <c r="C117" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="D117" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="118" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B118" s="31">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D118" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="119" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B119" s="31">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D119" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B120" s="31">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D120" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B121" s="31">
-        <v>53</v>
-      </c>
-      <c r="C121" s="28" t="s">
-        <v>143</v>
+        <v>52</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>141</v>
       </c>
       <c r="D121" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="122" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B122" s="31">
+        <v>53</v>
+      </c>
+      <c r="C122" s="28" t="s">
+        <v>143</v>
+      </c>
+      <c r="D122" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="123" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B123" s="31">
         <v>54</v>
       </c>
-      <c r="C122" s="28" t="s">
+      <c r="C123" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="D122" t="s">
+      <c r="D123" t="s">
         <v>146</v>
-      </c>
-    </row>
-    <row r="123" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B123" s="34">
-        <v>55</v>
-      </c>
-      <c r="C123" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="D123" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B124" s="34">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D124" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="125" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B125" s="34">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D125" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="126" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B126" s="34">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D126" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="127" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B127" s="34">
-        <v>59</v>
-      </c>
-      <c r="C127" s="28" t="s">
-        <v>151</v>
+        <v>58</v>
+      </c>
+      <c r="C127" s="8" t="s">
+        <v>150</v>
       </c>
       <c r="D127" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="128" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B128" s="34">
+        <v>59</v>
+      </c>
+      <c r="C128" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="D128" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B129" s="34">
         <v>60</v>
       </c>
-      <c r="C128" s="28" t="s">
+      <c r="C129" s="28" t="s">
         <v>152</v>
       </c>
-      <c r="D128" t="s">
+      <c r="D129" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A130" s="14" t="s">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="D130" t="s">
+      <c r="D131" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A132" s="14" t="s">
+      <c r="F131" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="D132" t="s">
+      <c r="D133" t="s">
         <v>188</v>
       </c>
-      <c r="F132" t="s">
+      <c r="F133" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A134" s="14" t="s">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="B134">
+      <c r="B135">
         <v>0</v>
       </c>
-      <c r="C134" t="s">
+      <c r="C135" t="s">
         <v>193</v>
       </c>
-      <c r="D134" t="s">
+      <c r="D135" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B135">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B136">
         <v>1</v>
       </c>
-      <c r="C135" t="s">
+      <c r="C136" t="s">
         <v>194</v>
       </c>
     </row>

</xml_diff>